<commit_message>
Management fee marketplace v0.2
</commit_message>
<xml_diff>
--- a/app/templates/report/recursos.xlsx
+++ b/app/templates/report/recursos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\oimbra\cotown\back\app\templates\report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\oimbra\custom\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB8468D0-6EDA-46F9-874C-A22F71491367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4156F3E6-5EF1-4A13-B476-E7883ED78FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Recursos" sheetId="37" r:id="rId1"/>
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">_Precios!$A$2:$N$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Recursos!$A$2:$BP$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Recursos!$A$2:$BQ$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Valoraciones!$A$2:$F$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="165">
   <si>
     <t>Code</t>
   </si>
@@ -540,6 +540,14 @@
   </si>
   <si>
     <t>Ical</t>
+  </si>
+  <si>
+    <t>M. Fee
+Market
+place</t>
+  </si>
+  <si>
+    <t>Management_fee_marketplace</t>
   </si>
 </sst>
 </file>
@@ -1184,51 +1192,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BR3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="24.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:BS3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="24.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="37.33203125" style="2" customWidth="1"/>
-    <col min="3" max="4" width="20.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="20.44140625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="29.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.88671875" style="2" customWidth="1"/>
-    <col min="13" max="13" width="14.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="12.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="21" width="12.33203125" style="2" customWidth="1"/>
-    <col min="22" max="29" width="9.5546875" style="2" customWidth="1"/>
-    <col min="30" max="30" width="53.6640625" style="2" customWidth="1"/>
-    <col min="31" max="31" width="10.6640625" style="2" customWidth="1"/>
-    <col min="32" max="32" width="30" style="2" customWidth="1"/>
-    <col min="33" max="33" width="24.6640625" style="2" customWidth="1"/>
-    <col min="34" max="34" width="11.88671875" style="31" customWidth="1"/>
-    <col min="35" max="36" width="11.5546875" style="2" customWidth="1"/>
-    <col min="37" max="38" width="17.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="10.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="11.5546875" style="2" customWidth="1"/>
-    <col min="41" max="41" width="10.6640625" style="2" customWidth="1"/>
-    <col min="42" max="42" width="14.109375" style="27" customWidth="1"/>
-    <col min="43" max="46" width="10.6640625" style="2" customWidth="1"/>
-    <col min="47" max="47" width="14.109375" style="27" customWidth="1"/>
-    <col min="48" max="52" width="11.88671875" style="2" customWidth="1"/>
-    <col min="53" max="55" width="17.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="56" max="57" width="15.44140625" style="2" customWidth="1"/>
-    <col min="58" max="59" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="12.6640625" style="2" customWidth="1"/>
-    <col min="62" max="63" width="13.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="64" max="67" width="16.88671875" style="2" customWidth="1"/>
-    <col min="68" max="68" width="20.5546875" style="2" customWidth="1"/>
-    <col min="69" max="69" width="93.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="5.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="71" max="16384" width="24.88671875" style="2"/>
+    <col min="1" max="2" width="37.28515625" style="2" customWidth="1"/>
+    <col min="3" max="4" width="20.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="20.42578125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="29.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.85546875" style="2" customWidth="1"/>
+    <col min="13" max="13" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="22" width="12.28515625" style="2" customWidth="1"/>
+    <col min="23" max="30" width="9.5703125" style="2" customWidth="1"/>
+    <col min="31" max="31" width="53.7109375" style="2" customWidth="1"/>
+    <col min="32" max="32" width="10.7109375" style="2" customWidth="1"/>
+    <col min="33" max="33" width="30" style="2" customWidth="1"/>
+    <col min="34" max="34" width="24.7109375" style="2" customWidth="1"/>
+    <col min="35" max="35" width="11.85546875" style="31" customWidth="1"/>
+    <col min="36" max="37" width="11.5703125" style="2" customWidth="1"/>
+    <col min="38" max="39" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="10.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="11.5703125" style="2" customWidth="1"/>
+    <col min="42" max="42" width="10.7109375" style="2" customWidth="1"/>
+    <col min="43" max="43" width="14.140625" style="27" customWidth="1"/>
+    <col min="44" max="47" width="10.7109375" style="2" customWidth="1"/>
+    <col min="48" max="48" width="14.140625" style="27" customWidth="1"/>
+    <col min="49" max="53" width="11.85546875" style="2" customWidth="1"/>
+    <col min="54" max="56" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="57" max="58" width="15.42578125" style="2" customWidth="1"/>
+    <col min="59" max="60" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="12.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="12.7109375" style="2" customWidth="1"/>
+    <col min="63" max="64" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="65" max="68" width="16.85546875" style="2" customWidth="1"/>
+    <col min="69" max="69" width="20.5703125" style="2" customWidth="1"/>
+    <col min="70" max="70" width="93.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="5.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="72" max="16384" width="24.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:70" s="1" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:71" s="1" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1289,155 +1297,158 @@
         <v>130</v>
       </c>
       <c r="V1" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="W1" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AB1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AC1" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AD1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AF1" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AG1" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="AG1" s="3" t="s">
+      <c r="AH1" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="AH1" s="28" t="s">
+      <c r="AI1" s="28" t="s">
         <v>101</v>
       </c>
-      <c r="AI1" s="21" t="s">
+      <c r="AJ1" s="21" t="s">
         <v>134</v>
       </c>
-      <c r="AJ1" s="21" t="s">
+      <c r="AK1" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="AK1" s="21" t="s">
+      <c r="AL1" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="AL1" s="21" t="s">
+      <c r="AM1" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="AM1" s="21" t="s">
+      <c r="AN1" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="AN1" s="21" t="s">
+      <c r="AO1" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="AO1" s="21" t="s">
+      <c r="AP1" s="21" t="s">
         <v>136</v>
       </c>
-      <c r="AP1" s="21" t="s">
+      <c r="AQ1" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="AQ1" s="21" t="s">
+      <c r="AR1" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="AR1" s="21" t="s">
+      <c r="AS1" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="AS1" s="21" t="s">
+      <c r="AT1" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="AT1" s="21" t="s">
+      <c r="AU1" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="AU1" s="21" t="s">
+      <c r="AV1" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="AV1" s="32" t="s">
+      <c r="AW1" s="32" t="s">
         <v>153</v>
       </c>
-      <c r="AW1" s="32" t="s">
+      <c r="AX1" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="AX1" s="32" t="s">
+      <c r="AY1" s="32" t="s">
         <v>155</v>
       </c>
-      <c r="AY1" s="32" t="s">
+      <c r="AZ1" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="AZ1" s="3" t="s">
+      <c r="BA1" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="BA1" s="3" t="s">
+      <c r="BB1" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="BB1" s="3" t="s">
+      <c r="BC1" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="BC1" s="3" t="s">
+      <c r="BD1" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="BD1" s="3" t="s">
+      <c r="BE1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="BE1" s="3" t="s">
+      <c r="BF1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="BF1" s="3" t="s">
+      <c r="BG1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="BG1" s="3" t="s">
+      <c r="BH1" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="BH1" s="3" t="s">
+      <c r="BI1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="BI1" s="3" t="s">
+      <c r="BJ1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="BJ1" s="3" t="s">
+      <c r="BK1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="BK1" s="3" t="s">
+      <c r="BL1" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="BL1" s="3" t="s">
+      <c r="BM1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="BM1" s="3" t="s">
+      <c r="BN1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="BN1" s="3" t="s">
+      <c r="BO1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="BO1" s="3" t="s">
+      <c r="BP1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="BP1" s="3" t="s">
+      <c r="BQ1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="BQ1" s="3" t="s">
+      <c r="BR1" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="BR1" s="1">
+      <c r="BS1" s="1">
         <f ca="1">IF(MONTH(TODAY())&gt;8,1+YEAR(TODAY()),YEAR(TODAY()))</f>
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
-    <row r="2" spans="1:70" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:71" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>67</v>
       </c>
@@ -1499,7 +1510,9 @@
       <c r="U2" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="V2" s="4"/>
+      <c r="V2" s="4" t="s">
+        <v>164</v>
+      </c>
       <c r="W2" s="4"/>
       <c r="X2" s="4"/>
       <c r="Y2" s="4"/>
@@ -1507,118 +1520,119 @@
       <c r="AA2" s="4"/>
       <c r="AB2" s="4"/>
       <c r="AC2" s="4"/>
-      <c r="AD2" s="4" t="s">
+      <c r="AD2" s="4"/>
+      <c r="AE2" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="AE2" s="4" t="s">
+      <c r="AF2" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="AF2" s="4" t="s">
+      <c r="AG2" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="AG2" s="4" t="s">
+      <c r="AH2" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="AH2" s="29" t="s">
+      <c r="AI2" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="AI2" s="4" t="s">
+      <c r="AJ2" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="AJ2" s="4" t="s">
+      <c r="AK2" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="AK2" s="4" t="s">
+      <c r="AL2" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="AL2" s="4" t="s">
+      <c r="AM2" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="AM2" s="4" t="s">
+      <c r="AN2" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="AN2" s="4" t="s">
+      <c r="AO2" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="AO2" s="4" t="s">
+      <c r="AP2" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="AP2" s="25" t="s">
+      <c r="AQ2" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="AQ2" s="4" t="s">
+      <c r="AR2" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="AR2" s="4" t="s">
+      <c r="AS2" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="AS2" s="4" t="s">
+      <c r="AT2" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="AT2" s="4" t="s">
+      <c r="AU2" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="AU2" s="25" t="s">
+      <c r="AV2" s="25" t="s">
         <v>152</v>
       </c>
-      <c r="AV2" s="4"/>
       <c r="AW2" s="4"/>
       <c r="AX2" s="4"/>
       <c r="AY2" s="4"/>
-      <c r="AZ2" s="4" t="s">
+      <c r="AZ2" s="4"/>
+      <c r="BA2" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="BA2" s="4" t="s">
+      <c r="BB2" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="BB2" s="4" t="s">
+      <c r="BC2" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="BC2" s="4" t="s">
+      <c r="BD2" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="BD2" s="4" t="s">
+      <c r="BE2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="BE2" s="4" t="s">
+      <c r="BF2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="BF2" s="4" t="s">
+      <c r="BG2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="BG2" s="4" t="s">
+      <c r="BH2" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="BH2" s="4" t="s">
+      <c r="BI2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="BI2" s="4" t="s">
+      <c r="BJ2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="BJ2" s="4" t="s">
+      <c r="BK2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="BK2" s="4" t="s">
+      <c r="BL2" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="BL2" s="4" t="s">
+      <c r="BM2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="BM2" s="4" t="s">
+      <c r="BN2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="BN2" s="4" t="s">
+      <c r="BO2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="BO2" s="4" t="s">
+      <c r="BP2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="BP2" s="4" t="s">
+      <c r="BQ2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="BQ2" s="4"/>
+      <c r="BR2" s="4"/>
     </row>
-    <row r="3" spans="1:70" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:71" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="9"/>
       <c r="C3" s="10"/>
@@ -1640,70 +1654,70 @@
       <c r="S3" s="10"/>
       <c r="T3" s="10"/>
       <c r="U3" s="10"/>
-      <c r="V3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BR$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($P3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+      <c r="V3" s="10"/>
+      <c r="W3" s="13">
+        <f ca="1">_xlfn.XLOOKUP($BS$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($P3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
-      <c r="W3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BR$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($P3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+      <c r="X3" s="13">
+        <f ca="1">_xlfn.XLOOKUP($BS$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($P3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
-      <c r="X3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BR$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($P3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+      <c r="Y3" s="13">
+        <f ca="1">_xlfn.XLOOKUP($BS$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($P3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
-      <c r="Y3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BR$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
+      <c r="Z3" s="13">
+        <f ca="1">_xlfn.XLOOKUP($BS$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
         <v>0</v>
       </c>
-      <c r="Z3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BR$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
+      <c r="AA3" s="13">
+        <f ca="1">_xlfn.XLOOKUP($BS$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
         <v>0</v>
       </c>
-      <c r="AA3" s="13">
-        <f t="shared" ref="AA3" ca="1" si="0">$V3+$Z3</f>
+      <c r="AB3" s="13">
+        <f t="shared" ref="AB3" ca="1" si="0">$W3+$AA3</f>
         <v>0</v>
       </c>
-      <c r="AB3" s="13">
-        <f t="shared" ref="AB3" ca="1" si="1">$W3+$Z3</f>
+      <c r="AC3" s="13">
+        <f t="shared" ref="AC3" ca="1" si="1">$X3+$AA3</f>
         <v>0</v>
       </c>
-      <c r="AC3" s="13">
-        <f t="shared" ref="AC3" ca="1" si="2">$X3+$Z3</f>
+      <c r="AD3" s="13">
+        <f t="shared" ref="AD3" ca="1" si="2">$Y3+$AA3</f>
         <v>0</v>
       </c>
-      <c r="AD3" s="20"/>
-      <c r="AE3" s="19" t="s">
+      <c r="AE3" s="20"/>
+      <c r="AF3" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="AF3" s="20"/>
-      <c r="AG3" s="17"/>
-      <c r="AH3" s="30"/>
-      <c r="AI3" s="22" t="s">
-        <v>96</v>
-      </c>
+      <c r="AG3" s="20"/>
+      <c r="AH3" s="17"/>
+      <c r="AI3" s="30"/>
       <c r="AJ3" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="AK3" s="24"/>
+      <c r="AK3" s="22" t="s">
+        <v>96</v>
+      </c>
       <c r="AL3" s="24"/>
       <c r="AM3" s="24"/>
-      <c r="AN3" s="22" t="s">
+      <c r="AN3" s="24"/>
+      <c r="AO3" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="AO3" s="23"/>
-      <c r="AP3" s="26"/>
-      <c r="AQ3" s="23"/>
+      <c r="AP3" s="23"/>
+      <c r="AQ3" s="26"/>
       <c r="AR3" s="23"/>
       <c r="AS3" s="23"/>
       <c r="AT3" s="23"/>
-      <c r="AU3" s="26"/>
-      <c r="AV3" s="33"/>
-      <c r="AW3" s="34"/>
+      <c r="AU3" s="23"/>
+      <c r="AV3" s="26"/>
+      <c r="AW3" s="33"/>
       <c r="AX3" s="34"/>
       <c r="AY3" s="34"/>
-      <c r="AZ3" s="18"/>
-      <c r="BA3" s="10"/>
+      <c r="AZ3" s="34"/>
+      <c r="BA3" s="18"/>
       <c r="BB3" s="10"/>
       <c r="BC3" s="10"/>
       <c r="BD3" s="10"/>
@@ -1720,10 +1734,11 @@
       <c r="BO3" s="10"/>
       <c r="BP3" s="10"/>
       <c r="BQ3" s="10"/>
+      <c r="BR3" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:BP3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="A3:BQ9988">
+  <autoFilter ref="A2:BQ3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="A3:BR9988">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>LEN($D3)=12</formula>
     </cfRule>
@@ -1737,12 +1752,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E1D64B2-929E-46C9-92E4-4B6A6392A32E}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="24.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="24.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.6640625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="20.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" style="2" customWidth="1"/>
     <col min="3" max="6" width="14" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="24.88671875" style="2"/>
+    <col min="7" max="16384" width="24.85546875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1811,17 +1826,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F063E8C-9C12-4A86-8416-6A77642A363A}">
   <dimension ref="A1:S3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="24.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="24.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="16.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="14.88671875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="24.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.88671875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="40.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="18" width="17.6640625" style="2" customWidth="1"/>
-    <col min="19" max="16384" width="24.88671875" style="2"/>
+    <col min="1" max="1" width="9.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.85546875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="40.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="18" width="17.7109375" style="2" customWidth="1"/>
+    <col min="19" max="16384" width="24.85546875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" s="1" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1958,12 +1973,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F48469C1-5DA9-43F7-A0B7-76DC91FAD532}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.33203125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="11.44140625" style="2"/>
+    <col min="1" max="1" width="7.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="11.42578125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2011,15 +2026,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101001BDC921D6C313740BA67D7760DC75571" ma:contentTypeVersion="9" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="ec6cd274e87ab0abf30bec2e834aaf15">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="220d4249-f262-4642-a86b-ff46de6e315d" xmlns:ns3="965e701d-44ad-4371-a199-8fefe953808c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e77808c4f084d99d477d3de919e85b9" ns2:_="" ns3:_="">
     <xsd:import namespace="220d4249-f262-4642-a86b-ff46de6e315d"/>
@@ -2216,6 +2222,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC650EC1-3E41-4FC6-BA6C-52921951A8DA}">
   <ds:schemaRefs>
@@ -2228,14 +2243,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91323775-37AE-44DC-8259-7FCDE5D849E0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2190EF49-E186-4D77-87E3-BC317999ED9E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2252,4 +2259,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91323775-37AE-44DC-8259-7FCDE5D849E0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>